<commit_message>
Adaptacion de ESTILOS A LA MARCA
</commit_message>
<xml_diff>
--- a/Fase 2/SIGMA_Burndown_Burnup.xlsx
+++ b/Fase 2/SIGMA_Burndown_Burnup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Capstone\SIGMA\Fase 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B9725D6-50AF-4EA9-BC2D-FA974C5D2531}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C1E2014-3556-455C-8DB2-3D632D139FFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resumen" sheetId="1" r:id="rId1"/>
@@ -87,7 +87,7 @@
     <t>Alcance total</t>
   </si>
   <si>
-    <t>751 puntos · 132 historias · 20 épicas</t>
+    <t>785 puntos · 138 historias · 20 épicas</t>
   </si>
   <si>
     <t>Versión</t>
@@ -222,7 +222,7 @@
     <t>Release burnup</t>
   </si>
   <si>
-    <t>Puntos completados acumulados del proyecto contra los 751 puntos del alcance total.</t>
+    <t>Puntos completados acumulados del proyecto contra los 785 puntos del alcance total.</t>
   </si>
   <si>
     <t>Permite proyectar la fecha de término: si la pendiente de la línea de completado se mantiene, el punto donde alcanzaría la línea de alcance es la fecha realista de cierre.</t>
@@ -662,11 +662,11 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -946,7 +946,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-B132-4762-B645-021A0F2657D1}"/>
+              <c16:uniqueId val="{00000000-B669-456A-9406-2265433BAD67}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1105,7 +1105,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-B132-4762-B645-021A0F2657D1}"/>
+              <c16:uniqueId val="{00000001-B669-456A-9406-2265433BAD67}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1546,7 +1546,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-EC1D-4FCC-8371-492022CFF2E3}"/>
+              <c16:uniqueId val="{00000000-E653-4D0B-8E1B-EEB9338F38D3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1696,7 +1696,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-EC1D-4FCC-8371-492022CFF2E3}"/>
+              <c16:uniqueId val="{00000001-E653-4D0B-8E1B-EEB9338F38D3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2128,7 +2128,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-FEEB-40E5-9A79-4E20A3027062}"/>
+              <c16:uniqueId val="{00000000-6CD0-479C-AE59-91C8F896EEE7}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2287,7 +2287,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-FEEB-40E5-9A79-4E20A3027062}"/>
+              <c16:uniqueId val="{00000001-6CD0-479C-AE59-91C8F896EEE7}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2728,7 +2728,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-166E-4F7D-9AFC-5722D9B2A42E}"/>
+              <c16:uniqueId val="{00000000-6DB3-4853-9621-C4623ED6620E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2878,7 +2878,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-166E-4F7D-9AFC-5722D9B2A42E}"/>
+              <c16:uniqueId val="{00000001-6DB3-4853-9621-C4623ED6620E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3259,13 +3259,13 @@
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0" formatCode="General">
-                  <c:v>751</c:v>
+                  <c:v>785</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>670</c:v>
+                  <c:v>704</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>561</c:v>
+                  <c:v>595</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>443</c:v>
@@ -3285,7 +3285,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-8FEB-43CE-BD95-2FDECDAB0C88}"/>
+              <c16:uniqueId val="{00000000-92A3-4581-A3FE-1CF741DA5207}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3393,25 +3393,25 @@
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0" formatCode="General">
-                  <c:v>751</c:v>
+                  <c:v>785</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>751</c:v>
+                  <c:v>785</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>751</c:v>
+                  <c:v>785</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>751</c:v>
+                  <c:v>785</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>751</c:v>
+                  <c:v>785</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>751</c:v>
+                  <c:v>785</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>751</c:v>
+                  <c:v>785</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3419,7 +3419,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-8FEB-43CE-BD95-2FDECDAB0C88}"/>
+              <c16:uniqueId val="{00000001-92A3-4581-A3FE-1CF741DA5207}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3834,7 +3834,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-5BC3-4248-A6E2-7C7B08511935}"/>
+              <c16:uniqueId val="{00000000-7B4E-4327-9294-CE769A78592D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3933,25 +3933,25 @@
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>751</c:v>
+                  <c:v>785</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>751</c:v>
+                  <c:v>785</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>751</c:v>
+                  <c:v>785</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>751</c:v>
+                  <c:v>785</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>751</c:v>
+                  <c:v>785</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>751</c:v>
+                  <c:v>785</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>751</c:v>
+                  <c:v>785</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3959,7 +3959,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-5BC3-4248-A6E2-7C7B08511935}"/>
+              <c16:uniqueId val="{00000001-7B4E-4327-9294-CE769A78592D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4401,7 +4401,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-9D41-4760-BC7C-E2BCC26D4EB9}"/>
+              <c16:uniqueId val="{00000000-4756-4B40-BAE7-BDBBCC90FBEF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4551,7 +4551,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-9D41-4760-BC7C-E2BCC26D4EB9}"/>
+              <c16:uniqueId val="{00000001-4756-4B40-BAE7-BDBBCC90FBEF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4977,7 +4977,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-172D-46DF-BB90-EFEEF28ECA74}"/>
+              <c16:uniqueId val="{00000000-1696-495A-A292-5B5EC59D1120}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5130,7 +5130,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-172D-46DF-BB90-EFEEF28ECA74}"/>
+              <c16:uniqueId val="{00000001-1696-495A-A292-5B5EC59D1120}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5565,7 +5565,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-91CC-401B-8B02-5B7B1E06DF15}"/>
+              <c16:uniqueId val="{00000000-A71D-46CD-A25D-1A2DA63B78D6}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5709,7 +5709,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-91CC-401B-8B02-5B7B1E06DF15}"/>
+              <c16:uniqueId val="{00000001-A71D-46CD-A25D-1A2DA63B78D6}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6135,7 +6135,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-90F3-45C0-86C9-8423F7431A84}"/>
+              <c16:uniqueId val="{00000000-38B5-4B13-8892-CDD8124B9A84}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6288,7 +6288,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-90F3-45C0-86C9-8423F7431A84}"/>
+              <c16:uniqueId val="{00000001-38B5-4B13-8892-CDD8124B9A84}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6723,7 +6723,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-5F19-4FE3-B914-D00D105EF2E8}"/>
+              <c16:uniqueId val="{00000000-E684-4B85-9399-16C0555CAD73}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6867,7 +6867,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-5F19-4FE3-B914-D00D105EF2E8}"/>
+              <c16:uniqueId val="{00000001-E684-4B85-9399-16C0555CAD73}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7299,7 +7299,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-8CAE-46D0-AE60-2209B4ACED66}"/>
+              <c16:uniqueId val="{00000000-25EE-4874-B7C9-ADCF44E5871A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7458,7 +7458,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-8CAE-46D0-AE60-2209B4ACED66}"/>
+              <c16:uniqueId val="{00000001-25EE-4874-B7C9-ADCF44E5871A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7899,7 +7899,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-F856-43EA-9790-3D37FCC22436}"/>
+              <c16:uniqueId val="{00000000-286F-40B1-AE87-C8422D694F32}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -8049,7 +8049,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-F856-43EA-9790-3D37FCC22436}"/>
+              <c16:uniqueId val="{00000001-286F-40B1-AE87-C8422D694F32}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -8481,7 +8481,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-4CEF-4B47-95A0-1B9E35DE508D}"/>
+              <c16:uniqueId val="{00000000-8ED3-48C1-92F4-2D36F04E19BB}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -8640,7 +8640,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-4CEF-4B47-95A0-1B9E35DE508D}"/>
+              <c16:uniqueId val="{00000001-8ED3-48C1-92F4-2D36F04E19BB}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -9804,7 +9804,7 @@
     <row r="21" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="7">
         <f>Release!$E$12</f>
-        <v>751</v>
+        <v>785</v>
       </c>
       <c r="C21" s="8">
         <f>SUM(Release!$F$6:$F$11)</f>
@@ -9812,7 +9812,7 @@
       </c>
       <c r="D21" s="8">
         <f>$B$21-$C$21</f>
-        <v>751</v>
+        <v>785</v>
       </c>
       <c r="E21" s="9">
         <f>IFERROR($C$21/$B$21,0)</f>
@@ -10194,7 +10194,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="43" t="s">
         <v>63</v>
       </c>
       <c r="B1" s="34"/>
@@ -10206,7 +10206,7 @@
       <c r="H1" s="34"/>
     </row>
     <row r="2" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="41" t="s">
         <v>64</v>
       </c>
       <c r="B2" s="34"/>
@@ -10712,7 +10712,7 @@
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A32" s="43" t="s">
+      <c r="A32" s="42" t="s">
         <v>87</v>
       </c>
       <c r="B32" s="34"/>
@@ -10745,17 +10745,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A25:B25"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A23:B23"/>
     <mergeCell ref="A32:H34"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A4:B4"/>
     <mergeCell ref="A27:H28"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A1:H1"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A25:B25"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.5"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
@@ -10787,7 +10787,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="43" t="s">
         <v>88</v>
       </c>
       <c r="B1" s="34"/>
@@ -10799,7 +10799,7 @@
       <c r="H1" s="34"/>
     </row>
     <row r="2" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="41" t="s">
         <v>89</v>
       </c>
       <c r="B2" s="34"/>
@@ -11269,16 +11269,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
-    <mergeCell ref="A26:H27"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A23:B23"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A1:H1"/>
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A1:H1"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A26:H27"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.5"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
@@ -11310,7 +11310,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="43" t="s">
         <v>90</v>
       </c>
       <c r="B1" s="34"/>
@@ -11322,7 +11322,7 @@
       <c r="H1" s="34"/>
     </row>
     <row r="2" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="41" t="s">
         <v>91</v>
       </c>
       <c r="B2" s="34"/>
@@ -11792,16 +11792,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
-    <mergeCell ref="A26:H27"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A23:B23"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A1:H1"/>
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A1:H1"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A26:H27"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.5"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
@@ -11833,7 +11833,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="43" t="s">
         <v>92</v>
       </c>
       <c r="B1" s="34"/>
@@ -11845,7 +11845,7 @@
       <c r="H1" s="34"/>
     </row>
     <row r="2" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="41" t="s">
         <v>93</v>
       </c>
       <c r="B2" s="34"/>
@@ -12347,16 +12347,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
-    <mergeCell ref="A25:B25"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A23:B23"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A4:B4"/>
     <mergeCell ref="A27:H28"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A1:H1"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A25:B25"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.5"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
@@ -12388,7 +12388,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="43" t="s">
         <v>94</v>
       </c>
       <c r="B1" s="34"/>
@@ -12400,7 +12400,7 @@
       <c r="H1" s="34"/>
     </row>
     <row r="2" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="41" t="s">
         <v>95</v>
       </c>
       <c r="B2" s="34"/>
@@ -12902,16 +12902,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
-    <mergeCell ref="A25:B25"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A23:B23"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A4:B4"/>
     <mergeCell ref="A27:H28"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A1:H1"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A25:B25"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.5"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
@@ -12943,7 +12943,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="43" t="s">
         <v>96</v>
       </c>
       <c r="B1" s="34"/>
@@ -12955,7 +12955,7 @@
       <c r="H1" s="34"/>
     </row>
     <row r="2" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="41" t="s">
         <v>97</v>
       </c>
       <c r="B2" s="34"/>
@@ -13457,16 +13457,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
-    <mergeCell ref="A25:B25"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A23:B23"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A4:B4"/>
     <mergeCell ref="A27:H28"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A1:H1"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A25:B25"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.5"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
@@ -13497,7 +13497,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="43" t="s">
         <v>98</v>
       </c>
       <c r="B1" s="34"/>
@@ -13509,7 +13509,7 @@
       <c r="H1" s="34"/>
     </row>
     <row r="2" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="41" t="s">
         <v>99</v>
       </c>
       <c r="B2" s="34"/>
@@ -13568,15 +13568,15 @@
         <v>0</v>
       </c>
       <c r="G5" s="11">
-        <f>751</f>
-        <v>751</v>
+        <f>785</f>
+        <v>785</v>
       </c>
       <c r="H5" s="11">
-        <v>751</v>
+        <v>785</v>
       </c>
       <c r="K5" s="26">
         <f t="shared" ref="K5:K11" si="0">$E$12</f>
-        <v>751</v>
+        <v>785</v>
       </c>
       <c r="L5" s="26">
         <f>$F$5</f>
@@ -13605,14 +13605,14 @@
       </c>
       <c r="G6" s="13">
         <f>$H$5-SUM($F$5:$F6)</f>
-        <v>751</v>
+        <v>785</v>
       </c>
       <c r="H6" s="13">
-        <v>670</v>
+        <v>704</v>
       </c>
       <c r="K6" s="26">
         <f t="shared" si="0"/>
-        <v>751</v>
+        <v>785</v>
       </c>
       <c r="L6" s="26">
         <f t="shared" ref="L6:L11" si="1">$L5+$F6</f>
@@ -13641,14 +13641,14 @@
       </c>
       <c r="G7" s="17">
         <f>$H$5-SUM($F$5:$F7)</f>
-        <v>751</v>
+        <v>785</v>
       </c>
       <c r="H7" s="17">
-        <v>561</v>
+        <v>595</v>
       </c>
       <c r="K7" s="26">
         <f t="shared" si="0"/>
-        <v>751</v>
+        <v>785</v>
       </c>
       <c r="L7" s="26">
         <f t="shared" si="1"/>
@@ -13669,7 +13669,7 @@
         <v>46308</v>
       </c>
       <c r="E8" s="11">
-        <v>118</v>
+        <v>152</v>
       </c>
       <c r="F8" s="13">
         <f>'Sprint 3'!$E$16</f>
@@ -13677,14 +13677,14 @@
       </c>
       <c r="G8" s="13">
         <f>$H$5-SUM($F$5:$F8)</f>
-        <v>751</v>
+        <v>785</v>
       </c>
       <c r="H8" s="13">
         <v>443</v>
       </c>
       <c r="K8" s="26">
         <f t="shared" si="0"/>
-        <v>751</v>
+        <v>785</v>
       </c>
       <c r="L8" s="26">
         <f t="shared" si="1"/>
@@ -13713,14 +13713,14 @@
       </c>
       <c r="G9" s="17">
         <f>$H$5-SUM($F$5:$F9)</f>
-        <v>751</v>
+        <v>785</v>
       </c>
       <c r="H9" s="17">
         <v>295</v>
       </c>
       <c r="K9" s="26">
         <f t="shared" si="0"/>
-        <v>751</v>
+        <v>785</v>
       </c>
       <c r="L9" s="26">
         <f t="shared" si="1"/>
@@ -13749,14 +13749,14 @@
       </c>
       <c r="G10" s="13">
         <f>$H$5-SUM($F$5:$F10)</f>
-        <v>751</v>
+        <v>785</v>
       </c>
       <c r="H10" s="13">
         <v>147</v>
       </c>
       <c r="K10" s="26">
         <f t="shared" si="0"/>
-        <v>751</v>
+        <v>785</v>
       </c>
       <c r="L10" s="26">
         <f t="shared" si="1"/>
@@ -13785,14 +13785,14 @@
       </c>
       <c r="G11" s="17">
         <f>$H$5-SUM($F$5:$F11)</f>
-        <v>751</v>
+        <v>785</v>
       </c>
       <c r="H11" s="17">
         <v>0</v>
       </c>
       <c r="K11" s="26">
         <f t="shared" si="0"/>
-        <v>751</v>
+        <v>785</v>
       </c>
       <c r="L11" s="26">
         <f t="shared" si="1"/>
@@ -13808,7 +13808,7 @@
       <c r="D12" s="19"/>
       <c r="E12" s="19">
         <f>SUM(E6:E11)</f>
-        <v>751</v>
+        <v>785</v>
       </c>
       <c r="F12" s="21">
         <f>SUM(F6:F11)</f>

</xml_diff>